<commit_message>
Atualizando lista de participantes no Excel
</commit_message>
<xml_diff>
--- a/bolao_atual.xlsx
+++ b/bolao_atual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a81d17a7f6589cb1/Python projects/Bolão/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF6DA5F2-DAC5-4A4E-BA59-00D82C013C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{DF6DA5F2-DAC5-4A4E-BA59-00D82C013C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A8C6D6D-B5A5-48E1-B03F-F8C90CF2036A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6E2B9C0F-DA98-462E-9B39-99169BF1CE84}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6E2B9C0F-DA98-462E-9B39-99169BF1CE84}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="91">
   <si>
     <t xml:space="preserve">Fláviana Roziriz </t>
   </si>
@@ -703,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E6D8180-E21A-492C-893E-09CB01200710}">
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="26.44140625" bestFit="1" customWidth="1"/>
@@ -1070,18 +1070,10 @@
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="3" t="s">
+      <c r="A46" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B46" s="3" t="s">
         <v>88</v>
       </c>
     </row>

</xml_diff>